<commit_message>
The files which created the results in the final paper
</commit_message>
<xml_diff>
--- a/Lander DB 251 redux (alt).xlsx
+++ b/Lander DB 251 redux (alt).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\conal\Desktop\PhD\EUCASS_2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cdepaor2\Desktop\EUCASS_2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33E69401-8EB1-42F9-ACD3-4A62A1B58040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF81D6BF-8632-48F7-BD66-613976C4E442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All Real Landers" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="Just models" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -73,9 +74,9 @@
     </comment>
     <comment ref="E1" authorId="1" shapeId="0" xr:uid="{14C96871-7C53-4D4A-88BE-E5819679F98D}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Commentaire à thread]
+Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
+Commentaire :
     bloc payload is an invented quantity to make 2stage manned landers, 1stage manned landers and 1stage unmanned landers comparable. it's definition is the following
 2stage manned landers: ascent stage mass
 1stage manned landers: landed mass
@@ -463,9 +464,9 @@
     </comment>
     <comment ref="E1" authorId="1" shapeId="0" xr:uid="{F43BA908-11C1-4486-9AC9-41BED78EF776}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Commentaire à thread]
+Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
+Commentaire :
     bloc payload is an invented quantity to make 2stage manned landers, 1stage manned landers and 1stage unmanned landers comparable. it's definition is the following
 2stage manned landers: ascent stage mass
 1stage manned landers: landed mass
@@ -902,9 +903,9 @@
     </comment>
     <comment ref="E1" authorId="1" shapeId="0" xr:uid="{B3F7CD30-2CE1-4425-828F-964D49209C6F}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Commentaire à thread]
+Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
+Commentaire :
     bloc payload is an invented quantity to make 2stage manned landers, 1stage manned landers and 1stage unmanned landers comparable. it's definition is the following
 2stage manned landers: ascent stage mass
 1stage manned landers: landed mass
@@ -1292,9 +1293,9 @@
     </comment>
     <comment ref="E1" authorId="1" shapeId="0" xr:uid="{1825771D-96A2-4E7C-B107-0F2AD72E57AE}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Commentaire à thread]
+Votre version d’Excel vous permet de lire ce commentaire à thread. Toutefois, les modifications qui y sont apportées seront supprimées si le fichier est ouvert dans une version plus récente d’Excel. En savoir plus : https://go.microsoft.com/fwlink/?linkid=870924
+Commentaire :
     bloc payload is an invented quantity to make 2stage manned landers, 1stage manned landers and 1stage unmanned landers comparable. it's definition is the following
 2stage manned landers: ascent stage mass
 1stage manned landers: landed mass
@@ -2209,20 +2210,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M30"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.73046875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.3984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.86328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.86328125" customWidth="1"/>
-    <col min="9" max="9" width="11.3984375" customWidth="1"/>
-    <col min="12" max="12" width="10.3984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.88671875" customWidth="1"/>
+    <col min="9" max="9" width="11.44140625" customWidth="1"/>
+    <col min="12" max="12" width="10.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2260,7 +2261,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="14">
         <v>1966</v>
       </c>
@@ -2302,7 +2303,7 @@
       </c>
       <c r="M2" s="4"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="8">
         <v>1966</v>
       </c>
@@ -2345,7 +2346,7 @@
       </c>
       <c r="M3" s="4"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <v>1966</v>
       </c>
@@ -2388,7 +2389,7 @@
       </c>
       <c r="M4" s="4"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="8">
         <v>1967</v>
       </c>
@@ -2430,7 +2431,7 @@
       </c>
       <c r="M5" s="4"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>1967</v>
       </c>
@@ -2472,7 +2473,7 @@
       </c>
       <c r="M6" s="4"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>1967</v>
       </c>
@@ -2514,7 +2515,7 @@
       </c>
       <c r="M7" s="4"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="8">
         <v>1968</v>
       </c>
@@ -2556,7 +2557,7 @@
       </c>
       <c r="M8" s="4"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>1969</v>
       </c>
@@ -2599,7 +2600,7 @@
       </c>
       <c r="M9" s="4"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="8">
         <v>1969</v>
       </c>
@@ -2642,7 +2643,7 @@
       </c>
       <c r="M10" s="4"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="8">
         <v>1970</v>
       </c>
@@ -2685,7 +2686,7 @@
       </c>
       <c r="M11" s="4"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>1970</v>
       </c>
@@ -2728,7 +2729,7 @@
       </c>
       <c r="M12" s="4"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>1970</v>
       </c>
@@ -2771,7 +2772,7 @@
       </c>
       <c r="M13" s="4"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
         <v>1971</v>
       </c>
@@ -2814,7 +2815,7 @@
       </c>
       <c r="M14" s="4"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>1971</v>
       </c>
@@ -2857,7 +2858,7 @@
       </c>
       <c r="M15" s="4"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>1972</v>
       </c>
@@ -2900,7 +2901,7 @@
       </c>
       <c r="M16" s="4"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" s="8">
         <v>1972</v>
       </c>
@@ -2943,7 +2944,7 @@
       </c>
       <c r="M17" s="4"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
         <v>1972</v>
       </c>
@@ -2986,7 +2987,7 @@
       </c>
       <c r="M18" s="4"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" s="5">
         <v>1973</v>
       </c>
@@ -3027,7 +3028,7 @@
       </c>
       <c r="M19" s="4"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" s="8">
         <v>1976</v>
       </c>
@@ -3070,7 +3071,7 @@
       </c>
       <c r="M20" s="4"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" s="5">
         <v>2013</v>
       </c>
@@ -3111,7 +3112,7 @@
       </c>
       <c r="M21" s="4"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" s="8">
         <v>2019</v>
       </c>
@@ -3152,7 +3153,7 @@
       </c>
       <c r="M22" s="4"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" s="5">
         <v>2019</v>
       </c>
@@ -3193,7 +3194,7 @@
       </c>
       <c r="M23" s="4"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" s="8">
         <v>2019</v>
       </c>
@@ -3234,7 +3235,7 @@
       </c>
       <c r="M24" s="4"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" s="5">
         <v>2020</v>
       </c>
@@ -3275,7 +3276,7 @@
       </c>
       <c r="M25" s="4"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" s="8">
         <v>2022</v>
       </c>
@@ -3316,7 +3317,7 @@
       </c>
       <c r="M26" s="4"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" s="8">
         <v>2023</v>
       </c>
@@ -3357,7 +3358,7 @@
       </c>
       <c r="M27" s="4"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" s="8">
         <v>2023</v>
       </c>
@@ -3397,7 +3398,7 @@
         <v>8.1105916056322808E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" s="5">
         <v>2024</v>
       </c>
@@ -3437,7 +3438,7 @@
         <v>9.5238095238095233E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" s="5">
         <v>2024</v>
       </c>
@@ -3504,9 +3505,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9B5FE63-1677-42A4-8B75-DD4C8D8979A4}">
   <dimension ref="A1:L32"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3544,7 +3545,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="11">
         <v>1966</v>
       </c>
@@ -3586,7 +3587,7 @@
         <v>0.12280701754385964</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="8">
         <v>1966</v>
       </c>
@@ -3628,7 +3629,7 @@
         <v>0.10540768905787917</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="8">
         <v>1966</v>
       </c>
@@ -3669,7 +3670,7 @@
         <v>0.11186440677966102</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="8">
         <v>1967</v>
       </c>
@@ -3710,7 +3711,7 @@
         <v>0.10855263157894737</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>1967</v>
       </c>
@@ -3751,7 +3752,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>1967</v>
       </c>
@@ -3792,7 +3793,7 @@
         <v>0.11036789297658862</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="8">
         <v>1968</v>
       </c>
@@ -3833,7 +3834,7 @@
         <v>0.10784313725490197</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="8">
         <v>1969</v>
       </c>
@@ -3875,7 +3876,7 @@
         <v>0.70328227571115975</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="5">
         <v>1969</v>
       </c>
@@ -3917,7 +3918,7 @@
         <v>0.70319568072377059</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>1970</v>
       </c>
@@ -3959,7 +3960,7 @@
         <v>0.68035768414671116</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>1970</v>
       </c>
@@ -4001,7 +4002,7 @@
         <v>0.39789473684210525</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
         <v>1970</v>
       </c>
@@ -4043,7 +4044,7 @@
         <v>0.27659574468085107</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>1971</v>
       </c>
@@ -4085,7 +4086,7 @@
         <v>0.64613933432152004</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="8">
         <v>1971</v>
       </c>
@@ -4127,7 +4128,7 @@
         <v>0.68773778167983612</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="8">
         <v>1972</v>
       </c>
@@ -4169,7 +4170,7 @@
         <v>0.64613933432152004</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="5">
         <v>1972</v>
       </c>
@@ -4211,7 +4212,7 @@
         <v>0.64613933432152004</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
         <v>1972</v>
       </c>
@@ -4253,7 +4254,7 @@
         <v>0.27659574468085107</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="5">
         <v>1973</v>
       </c>
@@ -4289,7 +4290,7 @@
         <v>0.45533769063180829</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="8">
         <v>1976</v>
       </c>
@@ -4331,7 +4332,7 @@
         <v>0.27393617021276595</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="5">
         <v>2013</v>
       </c>
@@ -4371,7 +4372,7 @@
         <v>0.12408759124087591</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="8">
         <v>2019</v>
       </c>
@@ -4411,7 +4412,7 @@
         <v>0.12408759124087591</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="5">
         <v>2019</v>
       </c>
@@ -4449,7 +4450,7 @@
         <v>4.1347626339969371E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="8">
         <v>2019</v>
       </c>
@@ -4489,7 +4490,7 @@
         <v>6.6622251832111927E-4</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" s="5">
         <v>2020</v>
       </c>
@@ -4529,7 +4530,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="8">
         <v>2022</v>
       </c>
@@ -4567,7 +4568,7 @@
         <v>0.12500000000000003</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="8">
         <v>2023</v>
       </c>
@@ -4605,7 +4606,7 @@
         <v>3.7499999999999999E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="8">
         <v>2023</v>
       </c>
@@ -4643,7 +4644,7 @@
         <v>8.1081081081081086E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="5">
         <v>2023</v>
       </c>
@@ -4670,7 +4671,7 @@
       <c r="J29" s="7"/>
       <c r="K29" s="3"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="5">
         <v>2024</v>
       </c>
@@ -4703,7 +4704,7 @@
       <c r="J30" s="10"/>
       <c r="K30" s="3"/>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" s="8">
         <v>2024</v>
       </c>
@@ -4730,7 +4731,7 @@
       <c r="J31" s="7"/>
       <c r="K31" s="3"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" s="5">
         <v>2024</v>
       </c>
@@ -4799,12 +4800,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DB6D447-256B-4552-8531-20A905B8B356}">
   <dimension ref="A1:L23"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.1328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4842,7 +4843,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="5">
         <v>1966</v>
       </c>
@@ -4884,7 +4885,7 @@
         <v>0.12280701754385964</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="8">
         <v>1966</v>
       </c>
@@ -4926,7 +4927,7 @@
         <v>0.10540768905787917</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="8">
         <v>1966</v>
       </c>
@@ -4967,7 +4968,7 @@
         <v>0.11186440677966102</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="8">
         <v>1967</v>
       </c>
@@ -5008,7 +5009,7 @@
         <v>0.10855263157894737</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>1967</v>
       </c>
@@ -5049,7 +5050,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>1967</v>
       </c>
@@ -5090,7 +5091,7 @@
         <v>0.11036789297658862</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="8">
         <v>1968</v>
       </c>
@@ -5131,7 +5132,7 @@
         <v>0.10784313725490197</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>1970</v>
       </c>
@@ -5173,7 +5174,7 @@
         <v>0.39789473684210525</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="8">
         <v>1970</v>
       </c>
@@ -5215,7 +5216,7 @@
         <v>0.27659574468085107</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>1972</v>
       </c>
@@ -5257,7 +5258,7 @@
         <v>0.27659574468085107</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>1973</v>
       </c>
@@ -5299,7 +5300,7 @@
         <v>0.45533769063180829</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
         <v>1976</v>
       </c>
@@ -5341,7 +5342,7 @@
         <v>0.27393617021276595</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>2013</v>
       </c>
@@ -5381,7 +5382,7 @@
         <v>0.12408759124087591</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="8">
         <v>2019</v>
       </c>
@@ -5421,7 +5422,7 @@
         <v>0.12408759124087591</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>2019</v>
       </c>
@@ -5459,7 +5460,7 @@
         <v>4.1347626339969371E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="8">
         <v>2019</v>
       </c>
@@ -5499,7 +5500,7 @@
         <v>6.6622251832111927E-4</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
         <v>2020</v>
       </c>
@@ -5539,7 +5540,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="8">
         <v>2022</v>
       </c>
@@ -5577,7 +5578,7 @@
         <v>0.12500000000000003</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="8">
         <v>2023</v>
       </c>
@@ -5615,7 +5616,7 @@
         <v>3.7499999999999999E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="8">
         <v>2023</v>
       </c>
@@ -5653,7 +5654,7 @@
         <v>8.1081081081081086E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="5">
         <v>2024</v>
       </c>
@@ -5693,7 +5694,7 @@
         <v>9.5238095238095233E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="5">
         <v>2024</v>
       </c>
@@ -5778,7 +5779,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21568D6A-64F0-4E55-9F6A-12E6ECCA0346}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -5787,9 +5788,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05661A04-FF2A-413A-B709-071725466C45}">
   <dimension ref="A1:L16"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5827,7 +5828,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="5">
         <v>1966</v>
       </c>
@@ -5869,7 +5870,7 @@
         <v>0.12280701754385964</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="8">
         <v>1966</v>
       </c>
@@ -5911,7 +5912,7 @@
         <v>0.10540768905787917</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="8">
         <v>1966</v>
       </c>
@@ -5952,7 +5953,7 @@
         <v>0.11186440677966102</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <v>1970</v>
       </c>
@@ -5994,7 +5995,7 @@
         <v>0.39789473684210525</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="8">
         <v>1970</v>
       </c>
@@ -6036,7 +6037,7 @@
         <v>0.27659574468085107</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>1973</v>
       </c>
@@ -6078,7 +6079,7 @@
         <v>0.45533769063180829</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="8">
         <v>1976</v>
       </c>
@@ -6120,7 +6121,7 @@
         <v>0.27393617021276595</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>2019</v>
       </c>
@@ -6158,7 +6159,7 @@
         <v>4.1347626339969371E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="8">
         <v>2019</v>
       </c>
@@ -6198,7 +6199,7 @@
         <v>6.6622251832111927E-4</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="5">
         <v>2020</v>
       </c>
@@ -6238,7 +6239,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="8">
         <v>2022</v>
       </c>
@@ -6276,7 +6277,7 @@
         <v>0.12500000000000003</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="8">
         <v>2023</v>
       </c>
@@ -6314,7 +6315,7 @@
         <v>3.7499999999999999E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="8">
         <v>2023</v>
       </c>
@@ -6352,7 +6353,7 @@
         <v>8.1081081081081086E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>2024</v>
       </c>
@@ -6392,7 +6393,7 @@
         <v>9.5238095238095233E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="5">
         <v>2024</v>
       </c>

</xml_diff>